<commit_message>
Add demo data validation and compatible uploads
</commit_message>
<xml_diff>
--- a/demo_urine_qac_masshunter.xlsx
+++ b/demo_urine_qac_masshunter.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,13 +37,21 @@
       <color rgb="002C3E50"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -58,10 +66,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,8 +444,27 @@
   <dimension ref="A1:U32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,6 +676,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -853,7 +888,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C10-DDAC</t>
+          <t>C10-DADMAC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1336,7 +1371,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C12-DDAC</t>
+          <t>C12-DADMAC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1681,7 +1716,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>C14-DDAC</t>
+          <t>C14-DADMAC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1888,7 +1923,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>C16-DDAC</t>
+          <t>C16-DADMAC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2095,7 +2130,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>C18-DDAC</t>
+          <t>C18-DADMAC</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2164,7 +2199,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>C8-10-DDAC</t>
+          <t>C8-10-DADMAC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2362,7 +2397,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>C8-DDAC</t>
+          <t>C8-DADMAC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2577,94 +2612,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>用途</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>仅用于网站功能演示，不用于科研结论</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>示例 MassHunter 原始定量结果，用于检查软件能否识别你的文件结构。</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>样本类型</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>尿液</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>导出值口径</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>有IS校正，换算因子=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>基质加标浓度</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>10 ppb（演示用）</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>SS加标浓度</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>d7-C12-BAC=4ppb，d9-C10-ATMAC=4ppb（演示用，非实验值）</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>应识别列</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>6 BLANK + 2 MS + 10 样品 + 2 SS</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>注意</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>此Demo为有IS校正口径。SS浓度为演示默认值。</t>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MassHunter 单位</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>ppb</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>默认内标校正</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>是；换算因子 = 1。若你的文件没有 IS 校正，请在软件中选择“否”。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>基质加标</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>F89-MS1、F90-MS2；基质加标浓度示例为 10 ppb。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>空白列</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>F91-BLANK1 至 F96-BLANK6，共 6 个。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>样品列</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>F1 至 F10，共 10 个；部分空单元格故意保留，用于检查 ND/缺失处理。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>IS</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>C12-BAC+COOH-d6、C12-BAC+OH-d3。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>d7-C12-BAC、d9-C10-ATMAC；默认各自加标浓度 4 ppb，可在软件中单独修改。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>命名规则</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>DDAC 在输出中统一显示为 DADMAC；链长和 BAC、DADMAC、ATMAC 类型会自动识别。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>使用方法</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>点击“加载 Demo 数据”，查看格式检查结果，再点击“开始处理”并下载结果。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close IS correction and reporting gaps
</commit_message>
<xml_diff>
--- a/demo_urine_qac_masshunter.xlsx
+++ b/demo_urine_qac_masshunter.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -676,8 +676,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -2599,6 +2597,69 @@
       </c>
       <c r="U32" t="n">
         <v>2.07200617756736</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>C8-PFAS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>499.0-&gt;80.0</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>10</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>